<commit_message>
Test data and Bugreport
</commit_message>
<xml_diff>
--- a/Project-01-Ecommerce-Manual-Testing/Bug report/bugreport.xlsx
+++ b/Project-01-Ecommerce-Manual-Testing/Bug report/bugreport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yashwanth y v\Desktop\QA portfolio\Project-01-Ecommerce-Manual-Testing\Bug report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32A8E1BD-D990-42C6-96B8-E20C992A1F01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E85CFCE-772E-44BE-B9CE-CE829597B7D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="71">
   <si>
     <t>Bug ID</t>
   </si>
@@ -161,6 +161,459 @@
   </si>
   <si>
     <t>Open</t>
+  </si>
+  <si>
+    <t>BUG-002</t>
+  </si>
+  <si>
+    <t>Products</t>
+  </si>
+  <si>
+    <t>Add to Cart button is not working for some products.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Open SauceDemo.2. Login using </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>error_user</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.3. Navigate to the Products page.4. Click </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Add to Cart</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> for different products.</t>
+    </r>
+  </si>
+  <si>
+    <t>All selected products should be added to the shopping cart.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Some products are added successfully, but </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Add to Cart</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> does not work for other products.</t>
+    </r>
+  </si>
+  <si>
+    <t>BUG-003</t>
+  </si>
+  <si>
+    <t>Shopping Cart</t>
+  </si>
+  <si>
+    <t>Remove button is not working for products added to the cart.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">2. Login using </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>error_user</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>3. Add a product to the cart.</t>
+  </si>
+  <si>
+    <t>4. Open the shopping cart.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">5. Click the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Remove</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> button.</t>
+    </r>
+  </si>
+  <si>
+    <t>The selected product should be removed from the shopping cart.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Clicking the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Remove</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> button does not remove the product from the shopping cart.</t>
+    </r>
+  </si>
+  <si>
+    <t>BUG-004</t>
+  </si>
+  <si>
+    <t>Sorting functionality is broken.</t>
+  </si>
+  <si>
+    <t>3. Navigate to the Products page.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">4. Click the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Sort</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> dropdown.</t>
+    </r>
+  </si>
+  <si>
+    <t>5. Select any sorting option (Name or Price).</t>
+  </si>
+  <si>
+    <t>Products should be sorted according to the selected sorting option.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The application displays the error message: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>"Sorting is broken! This error has been reported to Backtrace."</t>
+    </r>
+  </si>
+  <si>
+    <t>BUG-005</t>
+  </si>
+  <si>
+    <t>Product quantity cannot be increased in the shopping cart.</t>
+  </si>
+  <si>
+    <t>2. Login with any valid user.</t>
+  </si>
+  <si>
+    <t>5. Try to increase the product quantity.</t>
+  </si>
+  <si>
+    <t>The user should be able to increase the product quantity in the shopping cart.</t>
+  </si>
+  <si>
+    <t>The product quantity cannot be increased.</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>BUG-006</t>
+  </si>
+  <si>
+    <t>Checkout</t>
+  </si>
+  <si>
+    <t>Last Name field is cleared automatically after entering a value.</t>
+  </si>
+  <si>
+    <t>4. Proceed to Checkout.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">5. Enter valid values in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>First Name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Last Name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Postal Code</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>6. Observe the Last Name field.</t>
+  </si>
+  <si>
+    <t>The Last Name field should retain the entered value.</t>
+  </si>
+  <si>
+    <t>The Last Name field becomes empty even after a valid value is entered.</t>
+  </si>
+  <si>
+    <t>BUG-007</t>
+  </si>
+  <si>
+    <t>Checkout Overview</t>
+  </si>
+  <si>
+    <t>Finish button is not working on the Checkout Overview page.</t>
+  </si>
+  <si>
+    <t>4. Complete the checkout information.</t>
+  </si>
+  <si>
+    <t>5. Proceed to the Checkout Overview page.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">6. Click the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Finish</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> button.</t>
+    </r>
+  </si>
+  <si>
+    <t>The order should be completed successfully, and the Order Confirmation page should be displayed.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Clicking the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Finish</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> button does not complete the order or navigate to the Order Confirmation page.</t>
+    </r>
+  </si>
+  <si>
+    <t>BUG-008</t>
+  </si>
+  <si>
+    <t>Incorrect product images are displayed on the Products page.</t>
+  </si>
+  <si>
+    <t>4. Observe the product images.</t>
+  </si>
+  <si>
+    <t>Each product should display its correct corresponding image.</t>
+  </si>
+  <si>
+    <t>All product images are displayed as dog images instead of their respective product images.</t>
+  </si>
+  <si>
+    <r>
+      <t>2. Login using problem</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>_user</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -500,7 +953,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B107"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="48.88671875" customWidth="1"/>
@@ -597,10 +1050,671 @@
         <v>19</v>
       </c>
     </row>
+    <row r="14" spans="1:2">
+      <c r="A14" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="28.8">
+      <c r="A17" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="28.8">
+      <c r="A19" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" s="3"/>
+      <c r="B28" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" s="3"/>
+      <c r="B29" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" s="3"/>
+      <c r="B30" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" s="3"/>
+      <c r="B31" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="28.8">
+      <c r="A32" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="28.8">
+      <c r="A33" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" s="3"/>
+      <c r="B42" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" s="3"/>
+      <c r="B43" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" s="3"/>
+      <c r="B44" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" s="3"/>
+      <c r="B45" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="28.8">
+      <c r="A46" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="28.8">
+      <c r="A47" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" s="3"/>
+      <c r="B56" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" s="3"/>
+      <c r="B57" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" s="3"/>
+      <c r="B58" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2">
+      <c r="A59" s="3"/>
+      <c r="B59" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" ht="28.8">
+      <c r="A60" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2">
+      <c r="A61" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="A62" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2">
+      <c r="A63" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2">
+      <c r="A66" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2">
+      <c r="A67" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2">
+      <c r="A68" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2">
+      <c r="A69" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2">
+      <c r="A70" s="3"/>
+      <c r="B70" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2">
+      <c r="A71" s="3"/>
+      <c r="B71" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2">
+      <c r="A72" s="3"/>
+      <c r="B72" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2">
+      <c r="A73" s="3"/>
+      <c r="B73" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2">
+      <c r="A74" s="3"/>
+      <c r="B74" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" ht="28.8">
+      <c r="A76" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2">
+      <c r="A77" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2">
+      <c r="A78" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2">
+      <c r="A79" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2">
+      <c r="A83" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2">
+      <c r="A84" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2">
+      <c r="A85" s="3"/>
+      <c r="B85" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2">
+      <c r="A86" s="3"/>
+      <c r="B86" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2">
+      <c r="A87" s="3"/>
+      <c r="B87" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2">
+      <c r="A88" s="3"/>
+      <c r="B88" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2">
+      <c r="A89" s="3"/>
+      <c r="B89" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" ht="28.8">
+      <c r="A90" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" ht="28.8">
+      <c r="A91" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2">
+      <c r="A94" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2">
+      <c r="A96" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="A97" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2">
+      <c r="A98" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2">
+      <c r="A99" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2">
+      <c r="A100" s="3"/>
+      <c r="B100" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2">
+      <c r="A101" s="3"/>
+      <c r="B101" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2">
+      <c r="A102" s="3"/>
+      <c r="B102" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2">
+      <c r="A103" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" ht="28.8">
+      <c r="A104" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2">
+      <c r="A105" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2">
+      <c r="A106" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2">
+      <c r="A107" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="7">
+    <mergeCell ref="A84:A89"/>
+    <mergeCell ref="A99:A102"/>
     <mergeCell ref="A4:A7"/>
+    <mergeCell ref="A27:A31"/>
+    <mergeCell ref="A41:A45"/>
+    <mergeCell ref="A55:A59"/>
+    <mergeCell ref="A69:A74"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>